<commit_message>
Record: HRP and P36 site numbers back (1189410 on HRP, 1282487 on P36), 9515 -> 9527 verified
Andrew's site record (loading 10 Oct, photos 18 and 25 Sep) outranks the branch docket the 15 Oct fill used.
Put back through the page's own number controls with a backup first. Total unchanged at $147,017.32;
Baseplan 9968862 line 93 hire now joins HRP. AA 142514 untouched. Buildings workbook rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/buildings_charges_16Oct2026/GC500_Buildings_Charges_16Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/buildings_charges_16Oct2026/GC500_Buildings_Charges_16Oct2026.xlsx
@@ -695,15 +695,23 @@
           <t>Building 6m</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1189410</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9968862 / 93</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1426.07</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>145.74</v>
@@ -730,7 +738,13 @@
         <v>1603.78</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>1603.78</v>
+        <v>3029.85</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>1655.83</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>52.05</v>
       </c>
     </row>
     <row r="5">
@@ -2182,21 +2196,18 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1189410</t>
+          <t>1282487</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>9968862 / 93</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>1426.07</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>145.74</v>
@@ -2223,13 +2234,7 @@
         <v>1603.78</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>3029.85</v>
-      </c>
-      <c r="R26" s="2" t="n">
-        <v>1655.83</v>
-      </c>
-      <c r="S26" s="3" t="n">
-        <v>52.05</v>
+        <v>1603.78</v>
       </c>
     </row>
     <row r="27">

</xml_diff>